<commit_message>
Core_Data_추가, UI_Research 확장성 추가
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Research_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Research_Data.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmung\Desktop\Coding\Drill_Game\Assets\100_Data\XlsxFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Coding\Drill_Game\Assets\100_Data\XlsxFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFF3109-128D-43EF-A241-9F7D7C904CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2151" yWindow="686" windowWidth="18515" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2145" yWindow="690" windowWidth="18510" windowHeight="10740"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,12 +24,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>HOME2</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -91,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="97">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -113,10 +112,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>구리 생산량 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>구리 드릴</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -125,10 +120,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>철 생산량 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>철 드릴</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -157,10 +148,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Copper_UpProduce</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Copper_Discount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -173,10 +160,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Iron_UpProduce</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Iron_Discount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -193,13 +176,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>구리 자원들의 생산량이 증가합니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>철 자원들의 생산량이 증가합니다.</t>
-  </si>
-  <si>
     <t>구리 드릴로 업그레이드 합니다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -211,10 +187,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Gold_UpProduce</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Gold_Discount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -227,10 +199,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>금 생산량 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>금 효율 증가</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -247,10 +215,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Obsidian_UpProduce</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Obsidian_Discount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -263,10 +227,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>옵시디언 생산량 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>옵시디언 효율 증가</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -279,10 +239,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Tunstein_UpProduce</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Tunstein_Discount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -295,10 +251,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>텅스텐 생산량 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>텅스텐 효율 증가</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -307,18 +259,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>금 자원들의 생산량이 증가합니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>금 드릴로 업그레이드 합니다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>옵시디언 자원들의 생산량이 증가합니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>옵시디언 시설을 설치할 수 있게 됩니다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -331,10 +275,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>텅스텐 자원들의 생산량이 증가합니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>텅스텐 드릴로 업그레이드 합니다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -343,10 +283,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Titanium_UpProduce</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Titanium_Discount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -359,10 +295,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>티타늄 생산량 증가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>티타늄 효율 증가</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -375,10 +307,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>티타늄 자원들의 생산량이 증가합니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>티타늄 드릴로 업그레이드 합니다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -404,13 +332,154 @@
   </si>
   <si>
     <t>티타늄 자원을 소모할 때 소모량이 감소합니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Copper_Lv2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>구리 테크 Lv.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.2의 구리 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Copper_Lv3</t>
+  </si>
+  <si>
+    <t>구리 테크 Lv.3</t>
+  </si>
+  <si>
+    <t>Lv.3의 구리 시설을 설치할 수 있게 됩니다.</t>
+  </si>
+  <si>
+    <t>Iron_Lv2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Iron_Lv3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>철 테크 Lv.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>철 테크 Lv.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.2의 철 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.3의 철 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>금 테크 Lv.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>금 테크 Lv.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gold_Lv2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gold_Lv3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.2의 금 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.3의 금 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Obsidian_Lv2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Obsidian_Lv3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>옵시디언 테크 Lv.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>옵시디언 테크 Lv.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.2의 옵시디언 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.3의 옵시디언 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>텅스텐 테크 Lv.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>텅스텐 테크 Lv.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tunstein_Lv2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tunstein_Lv3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.2의 텅스텐 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.3의 텅스텐 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Titanium_Lv2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Titanium_Lv3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 테크 Lv.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 테크 Lv.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.2의 티타늄 시설을 설치할 수 있게 됩니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lv.3의 티타늄 시설을 설치할 수 있게 됩니다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -487,17 +556,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표1" displayName="표1" ref="A1:H25" totalsRowShown="0">
-  <autoFilter ref="A1:H25" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="표1" displayName="표1" ref="A1:H31" totalsRowShown="0">
+  <autoFilter ref="A1:H31"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DisplayName"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Desc"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="ResearchAmount"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="InputItemPerTickId"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="InputItemPerTickCount"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="RequireResearchId"/>
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="7" name="Name"/>
+    <tableColumn id="2" name="DisplayName"/>
+    <tableColumn id="8" name="Desc"/>
+    <tableColumn id="3" name="ResearchAmount"/>
+    <tableColumn id="5" name="InputItemPerTickId"/>
+    <tableColumn id="6" name="InputItemPerTickCount"/>
+    <tableColumn id="4" name="RequireResearchId"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -765,57 +834,57 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.75" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="38.140625" customWidth="1"/>
-    <col min="5" max="5" width="17.640625" customWidth="1"/>
-    <col min="6" max="6" width="20.35546875" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="38.125" customWidth="1"/>
+    <col min="5" max="5" width="17.625" customWidth="1"/>
+    <col min="6" max="6" width="20.375" customWidth="1"/>
+    <col min="7" max="7" width="17.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>30001</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E2">
         <v>50</v>
@@ -827,18 +896,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>30002</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="E3">
         <v>100</v>
@@ -853,18 +922,18 @@
         <v>30001</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>30003</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E4">
         <v>100</v>
@@ -879,18 +948,18 @@
         <v>30001</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>30004</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E5">
         <v>100</v>
@@ -905,21 +974,21 @@
         <v>30001</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>30005</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E6">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F6">
         <v>1004</v>
@@ -931,44 +1000,44 @@
         <v>30001</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>30006</v>
       </c>
       <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
       <c r="E7">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="F7">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>30002</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>30007</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E8">
         <v>200</v>
@@ -980,21 +1049,21 @@
         <v>2</v>
       </c>
       <c r="H8">
-        <v>30002</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30006</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>30008</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="E9">
         <v>200</v>
@@ -1006,24 +1075,24 @@
         <v>2</v>
       </c>
       <c r="H9">
-        <v>30002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30006</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>30009</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E10">
-        <v>750</v>
+        <v>200</v>
       </c>
       <c r="F10">
         <v>1006</v>
@@ -1032,73 +1101,73 @@
         <v>2</v>
       </c>
       <c r="H10">
-        <v>30005</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30006</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>30010</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="E11">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="F11">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="G11">
         <v>2</v>
       </c>
       <c r="H11">
-        <v>30009</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30006</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>30011</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
+        <v>29</v>
       </c>
       <c r="E12">
-        <v>400</v>
+        <v>750</v>
       </c>
       <c r="F12">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="G12">
         <v>2</v>
       </c>
       <c r="H12">
-        <v>30009</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30006</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>30012</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="E13">
         <v>400</v>
@@ -1110,24 +1179,24 @@
         <v>2</v>
       </c>
       <c r="H13">
-        <v>30009</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30011</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>30013</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="E14">
-        <v>2000</v>
+        <v>400</v>
       </c>
       <c r="F14">
         <v>1008</v>
@@ -1136,102 +1205,102 @@
         <v>2</v>
       </c>
       <c r="H14">
-        <v>30009</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30011</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>30014</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E15">
         <v>400</v>
       </c>
       <c r="F15">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="G15">
         <v>2</v>
       </c>
       <c r="H15">
-        <v>30013</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30011</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>30015</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="E16">
         <v>400</v>
       </c>
       <c r="F16">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="G16">
         <v>2</v>
       </c>
       <c r="H16">
-        <v>30013</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30011</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>30016</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="E17">
-        <v>400</v>
+        <v>2000</v>
       </c>
       <c r="F17">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>30013</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30011</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>30017</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="E18">
-        <v>4000</v>
+        <v>400</v>
       </c>
       <c r="F18">
         <v>1010</v>
@@ -1240,131 +1309,131 @@
         <v>2</v>
       </c>
       <c r="H18">
-        <v>30013</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30016</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>30018</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="E19">
         <v>400</v>
       </c>
       <c r="F19">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="G19">
         <v>2</v>
       </c>
       <c r="H19">
-        <v>30017</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30016</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>30019</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="E20">
         <v>400</v>
       </c>
       <c r="F20">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>30017</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30016</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>30020</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="D21" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="E21">
         <v>400</v>
       </c>
       <c r="F21">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
       <c r="H21">
-        <v>30017</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30016</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>30021</v>
       </c>
       <c r="B22" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="D22" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="E22">
-        <v>6000</v>
+        <v>4000</v>
       </c>
       <c r="F22">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="G22">
         <v>2</v>
       </c>
       <c r="H22">
-        <v>30017</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>30016</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>30022</v>
       </c>
       <c r="B23" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="C23" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="D23" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="E23">
         <v>400</v>
       </c>
       <c r="F23">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="G23">
         <v>2</v>
@@ -1373,24 +1442,24 @@
         <v>30021</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>30023</v>
       </c>
       <c r="B24" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D24" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="E24">
         <v>400</v>
       </c>
       <c r="F24">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="G24">
         <v>2</v>
@@ -1399,30 +1468,186 @@
         <v>30021</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>30024</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E25">
         <v>400</v>
       </c>
       <c r="F25">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="G25">
         <v>2</v>
       </c>
       <c r="H25">
         <v>30021</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>30025</v>
+      </c>
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" t="s">
+        <v>41</v>
+      </c>
+      <c r="D26" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26">
+        <v>400</v>
+      </c>
+      <c r="F26">
+        <v>1012</v>
+      </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
+      <c r="H26">
+        <v>30021</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>30026</v>
+      </c>
+      <c r="B27" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27">
+        <v>6000</v>
+      </c>
+      <c r="F27">
+        <v>1012</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+      <c r="H27">
+        <v>30021</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>30027</v>
+      </c>
+      <c r="B28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" t="s">
+        <v>95</v>
+      </c>
+      <c r="E28">
+        <v>400</v>
+      </c>
+      <c r="F28">
+        <v>1014</v>
+      </c>
+      <c r="G28">
+        <v>2</v>
+      </c>
+      <c r="H28">
+        <v>30026</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>30028</v>
+      </c>
+      <c r="B29" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" t="s">
+        <v>94</v>
+      </c>
+      <c r="D29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E29">
+        <v>400</v>
+      </c>
+      <c r="F29">
+        <v>1014</v>
+      </c>
+      <c r="G29">
+        <v>2</v>
+      </c>
+      <c r="H29">
+        <v>30026</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>30029</v>
+      </c>
+      <c r="B30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" t="s">
+        <v>60</v>
+      </c>
+      <c r="E30">
+        <v>400</v>
+      </c>
+      <c r="F30">
+        <v>1014</v>
+      </c>
+      <c r="G30">
+        <v>2</v>
+      </c>
+      <c r="H30">
+        <v>30026</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>30030</v>
+      </c>
+      <c r="B31" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" t="s">
+        <v>54</v>
+      </c>
+      <c r="E31">
+        <v>400</v>
+      </c>
+      <c r="F31">
+        <v>1014</v>
+      </c>
+      <c r="G31">
+        <v>2</v>
+      </c>
+      <c r="H31">
+        <v>30026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>